<commit_message>
final data updates. only change is adding the water components data sheet correctly.
</commit_message>
<xml_diff>
--- a/intermediate/dashboard_output_poverty.xlsx
+++ b/intermediate/dashboard_output_poverty.xlsx
@@ -457,7 +457,7 @@
         </is>
       </c>
       <c r="H2">
-        <v>-0.9176107614463774</v>
+        <v>-0.9117363939281745</v>
       </c>
       <c r="I2">
         <v>2025</v>
@@ -482,7 +482,7 @@
         <v>2015</v>
       </c>
       <c r="O2">
-        <v>28.27</v>
+        <v>28.175</v>
       </c>
     </row>
     <row r="3">
@@ -514,7 +514,7 @@
         <v>2027</v>
       </c>
       <c r="H3">
-        <v>2.641415145214415</v>
+        <v>2.866193274227115</v>
       </c>
       <c r="I3">
         <v>2025</v>
@@ -539,7 +539,7 @@
         <v>2015</v>
       </c>
       <c r="O3">
-        <v>7.605</v>
+        <v>7.81</v>
       </c>
     </row>
     <row r="4">
@@ -638,7 +638,7 @@
         <v>2015</v>
       </c>
       <c r="O5">
-        <v>0.71</v>
+        <v>0.74</v>
       </c>
     </row>
     <row r="6">
@@ -692,7 +692,7 @@
         <v>2015</v>
       </c>
       <c r="O6">
-        <v>1.825</v>
+        <v>1.92</v>
       </c>
     </row>
     <row r="7">
@@ -746,7 +746,7 @@
         <v>2015</v>
       </c>
       <c r="O7">
-        <v>0.4</v>
+        <v>0.42</v>
       </c>
     </row>
     <row r="8">
@@ -800,7 +800,7 @@
         <v>2015</v>
       </c>
       <c r="O8">
-        <v>0.465</v>
+        <v>0.485</v>
       </c>
     </row>
     <row r="9">
@@ -874,10 +874,10 @@
         </is>
       </c>
       <c r="G10">
-        <v>2646</v>
+        <v>2653</v>
       </c>
       <c r="H10">
-        <v>0.2082205704847212</v>
+        <v>0.2111460517120889</v>
       </c>
       <c r="I10">
         <v>2025</v>
@@ -902,7 +902,7 @@
         <v>2015</v>
       </c>
       <c r="O10">
-        <v>69.39</v>
+        <v>69.47499999999999</v>
       </c>
     </row>
     <row r="11">
@@ -976,10 +976,10 @@
         </is>
       </c>
       <c r="G12">
-        <v>2044</v>
+        <v>2045</v>
       </c>
       <c r="H12">
-        <v>2.835998074157635</v>
+        <v>2.798301147486171</v>
       </c>
       <c r="I12">
         <v>2025</v>
@@ -1004,7 +1004,7 @@
         <v>2015</v>
       </c>
       <c r="O12">
-        <v>33.79</v>
+        <v>33.725</v>
       </c>
     </row>
     <row r="13">
@@ -1033,10 +1033,10 @@
         </is>
       </c>
       <c r="G13">
-        <v>2054</v>
+        <v>2055</v>
       </c>
       <c r="H13">
-        <v>2.455004261448406</v>
+        <v>2.451171891069151</v>
       </c>
       <c r="I13">
         <v>2025</v>
@@ -1061,7 +1061,7 @@
         <v>2015</v>
       </c>
       <c r="O13">
-        <v>44.86499999999999</v>
+        <v>44.88500000000001</v>
       </c>
     </row>
     <row r="14">
@@ -1090,10 +1090,10 @@
         </is>
       </c>
       <c r="G14">
-        <v>2043</v>
+        <v>2044</v>
       </c>
       <c r="H14">
-        <v>1.438383992335636</v>
+        <v>1.506458799858635</v>
       </c>
       <c r="I14">
         <v>2025</v>
@@ -1118,7 +1118,7 @@
         <v>2015</v>
       </c>
       <c r="O14">
-        <v>10.48</v>
+        <v>10.635</v>
       </c>
     </row>
     <row r="15">
@@ -1150,7 +1150,7 @@
         <v>2017</v>
       </c>
       <c r="H15">
-        <v>3.758774625357441</v>
+        <v>4.190405419743658</v>
       </c>
       <c r="I15">
         <v>2025</v>
@@ -1175,7 +1175,7 @@
         <v>2015</v>
       </c>
       <c r="O15">
-        <v>2.92</v>
+        <v>3.055</v>
       </c>
     </row>
     <row r="16">
@@ -1229,7 +1229,7 @@
         <v>2015</v>
       </c>
       <c r="O16">
-        <v>0.535</v>
+        <v>0.555</v>
       </c>
     </row>
     <row r="17">
@@ -1328,7 +1328,7 @@
         <v>2015</v>
       </c>
       <c r="O18">
-        <v>0.585</v>
+        <v>0.625</v>
       </c>
     </row>
     <row r="19">
@@ -1360,7 +1360,7 @@
         <v>2026</v>
       </c>
       <c r="H19">
-        <v>1.49683131987066</v>
+        <v>1.652047055504283</v>
       </c>
       <c r="I19">
         <v>2025</v>
@@ -1385,7 +1385,7 @@
         <v>2015</v>
       </c>
       <c r="O19">
-        <v>3.97</v>
+        <v>4.135</v>
       </c>
     </row>
     <row r="20">
@@ -1417,7 +1417,7 @@
         <v>2025</v>
       </c>
       <c r="H20">
-        <v>1.378935237691968</v>
+        <v>1.525656236178682</v>
       </c>
       <c r="I20">
         <v>2025</v>
@@ -1442,7 +1442,7 @@
         <v>2015</v>
       </c>
       <c r="O20">
-        <v>3.44</v>
+        <v>3.595</v>
       </c>
     </row>
     <row r="21">
@@ -1496,7 +1496,7 @@
         <v>2015</v>
       </c>
       <c r="O21">
-        <v>1.015</v>
+        <v>1.065</v>
       </c>
     </row>
     <row r="22">
@@ -1570,10 +1570,10 @@
         </is>
       </c>
       <c r="G23">
-        <v>2470</v>
+        <v>2504</v>
       </c>
       <c r="H23">
-        <v>0.1117796610169478</v>
+        <v>0.1106214689265556</v>
       </c>
       <c r="I23">
         <v>2025</v>
@@ -1598,7 +1598,7 @@
         <v>2015</v>
       </c>
       <c r="O23">
-        <v>15.025</v>
+        <v>15.05</v>
       </c>
     </row>
     <row r="24">
@@ -1627,10 +1627,10 @@
         </is>
       </c>
       <c r="G24">
-        <v>2127</v>
+        <v>2128</v>
       </c>
       <c r="H24">
-        <v>1.150632994899395</v>
+        <v>1.164879169017146</v>
       </c>
       <c r="I24">
         <v>2025</v>
@@ -1655,7 +1655,7 @@
         <v>2015</v>
       </c>
       <c r="O24">
-        <v>67.69</v>
+        <v>67.77500000000001</v>
       </c>
     </row>
     <row r="25">
@@ -1808,7 +1808,7 @@
         <v>2015</v>
       </c>
       <c r="O27">
-        <v>0.465</v>
+        <v>0.485</v>
       </c>
     </row>
     <row r="28">
@@ -1882,10 +1882,10 @@
         </is>
       </c>
       <c r="G29">
-        <v>2050</v>
+        <v>2052</v>
       </c>
       <c r="H29">
-        <v>1.716316350985153</v>
+        <v>1.702001567900291</v>
       </c>
       <c r="I29">
         <v>2025</v>
@@ -1910,7 +1910,7 @@
         <v>2015</v>
       </c>
       <c r="O29">
-        <v>19.785</v>
+        <v>19.685</v>
       </c>
     </row>
     <row r="30">
@@ -1939,7 +1939,7 @@
         </is>
       </c>
       <c r="H30">
-        <v>-0.1149253731343265</v>
+        <v>-0.1131287297527706</v>
       </c>
       <c r="I30">
         <v>2025</v>
@@ -1964,7 +1964,7 @@
         <v>2015</v>
       </c>
       <c r="O30">
-        <v>20.76</v>
+        <v>20.655</v>
       </c>
     </row>
     <row r="31">
@@ -1993,10 +1993,10 @@
         </is>
       </c>
       <c r="G31">
-        <v>2215</v>
+        <v>2218</v>
       </c>
       <c r="H31">
-        <v>0.7515743144798733</v>
+        <v>0.7610213859689182</v>
       </c>
       <c r="I31">
         <v>2025</v>
@@ -2021,7 +2021,7 @@
         <v>2015</v>
       </c>
       <c r="O31">
-        <v>79.76000000000001</v>
+        <v>79.815</v>
       </c>
     </row>
     <row r="32">
@@ -2050,7 +2050,7 @@
         </is>
       </c>
       <c r="H32">
-        <v>-1.727786005183268</v>
+        <v>-1.726990003702332</v>
       </c>
       <c r="I32">
         <v>2025</v>
@@ -2075,7 +2075,7 @@
         <v>2015</v>
       </c>
       <c r="O32">
-        <v>31.485</v>
+        <v>31.42</v>
       </c>
     </row>
     <row r="33">
@@ -2104,10 +2104,10 @@
         </is>
       </c>
       <c r="G33">
-        <v>2059</v>
+        <v>2060</v>
       </c>
       <c r="H33">
-        <v>0.672251304047532</v>
+        <v>0.720256516332222</v>
       </c>
       <c r="I33">
         <v>2025</v>
@@ -2132,7 +2132,7 @@
         <v>2015</v>
       </c>
       <c r="O33">
-        <v>6.735</v>
+        <v>6.945</v>
       </c>
     </row>
     <row r="34">
@@ -2164,7 +2164,7 @@
         <v>2031</v>
       </c>
       <c r="H34">
-        <v>1.692508701805593</v>
+        <v>1.841648752968197</v>
       </c>
       <c r="I34">
         <v>2025</v>
@@ -2189,7 +2189,7 @@
         <v>2015</v>
       </c>
       <c r="O34">
-        <v>6.100000000000001</v>
+        <v>6.295</v>
       </c>
     </row>
     <row r="35">
@@ -2218,10 +2218,10 @@
         </is>
       </c>
       <c r="G35">
-        <v>2049</v>
+        <v>2050</v>
       </c>
       <c r="H35">
-        <v>1.173022896545967</v>
+        <v>1.228257519346428</v>
       </c>
       <c r="I35">
         <v>2025</v>
@@ -2246,7 +2246,7 @@
         <v>2015</v>
       </c>
       <c r="O35">
-        <v>10.015</v>
+        <v>10.185</v>
       </c>
     </row>
     <row r="36">
@@ -2300,7 +2300,7 @@
         <v>2015</v>
       </c>
       <c r="O36">
-        <v>1.58</v>
+        <v>1.655</v>
       </c>
     </row>
     <row r="37">
@@ -2464,10 +2464,10 @@
         </is>
       </c>
       <c r="G40">
-        <v>2056</v>
+        <v>2058</v>
       </c>
       <c r="H40">
-        <v>1.578289175421682</v>
+        <v>1.553491061504082</v>
       </c>
       <c r="I40">
         <v>2025</v>
@@ -2492,7 +2492,7 @@
         <v>2015</v>
       </c>
       <c r="O40">
-        <v>22.555</v>
+        <v>22.44</v>
       </c>
     </row>
     <row r="41">
@@ -2591,7 +2591,7 @@
         <v>2015</v>
       </c>
       <c r="O42">
-        <v>1.265</v>
+        <v>1.33</v>
       </c>
     </row>
     <row r="43">
@@ -2668,7 +2668,7 @@
         <v>2029</v>
       </c>
       <c r="H44">
-        <v>0.7864907980736149</v>
+        <v>0.8691987463001396</v>
       </c>
       <c r="I44">
         <v>2025</v>
@@ -2693,7 +2693,7 @@
         <v>2015</v>
       </c>
       <c r="O44">
-        <v>3.05</v>
+        <v>3.185</v>
       </c>
     </row>
     <row r="45">
@@ -2747,7 +2747,7 @@
         <v>2015</v>
       </c>
       <c r="O45">
-        <v>0.4</v>
+        <v>0.42</v>
       </c>
     </row>
     <row r="46">
@@ -2801,7 +2801,7 @@
         <v>2015</v>
       </c>
       <c r="O46">
-        <v>0.71</v>
+        <v>0.74</v>
       </c>
     </row>
     <row r="47">
@@ -2855,7 +2855,7 @@
         <v>2015</v>
       </c>
       <c r="O47">
-        <v>0.465</v>
+        <v>0.485</v>
       </c>
     </row>
     <row r="48">
@@ -2884,7 +2884,7 @@
         </is>
       </c>
       <c r="H48">
-        <v>-1.158337403581473</v>
+        <v>-1.149591200789831</v>
       </c>
       <c r="I48">
         <v>2025</v>
@@ -2909,7 +2909,7 @@
         <v>2015</v>
       </c>
       <c r="O48">
-        <v>26.22</v>
+        <v>26.11</v>
       </c>
     </row>
     <row r="49">
@@ -2986,7 +2986,7 @@
         <v>2024</v>
       </c>
       <c r="H50">
-        <v>1.949982668522009</v>
+        <v>2.158599959122407</v>
       </c>
       <c r="I50">
         <v>2025</v>
@@ -3011,7 +3011,7 @@
         <v>2015</v>
       </c>
       <c r="O50">
-        <v>3.705</v>
+        <v>3.86</v>
       </c>
     </row>
     <row r="51">
@@ -3085,10 +3085,10 @@
         </is>
       </c>
       <c r="G52">
-        <v>2236</v>
+        <v>2252</v>
       </c>
       <c r="H52">
-        <v>0.2649206349206338</v>
+        <v>0.2599344405594423</v>
       </c>
       <c r="I52">
         <v>2025</v>
@@ -3113,7 +3113,7 @@
         <v>2015</v>
       </c>
       <c r="O52">
-        <v>19.16</v>
+        <v>19.08</v>
       </c>
     </row>
     <row r="53">
@@ -3142,7 +3142,7 @@
         </is>
       </c>
       <c r="H53">
-        <v>-0.7160146075974267</v>
+        <v>-0.7921599955771768</v>
       </c>
       <c r="I53">
         <v>2025</v>
@@ -3167,7 +3167,7 @@
         <v>2015</v>
       </c>
       <c r="O53">
-        <v>2.275</v>
+        <v>2.38</v>
       </c>
     </row>
     <row r="54">
@@ -3221,7 +3221,7 @@
         <v>2015</v>
       </c>
       <c r="O54">
-        <v>0.21</v>
+        <v>0.22</v>
       </c>
     </row>
     <row r="55">
@@ -3253,7 +3253,7 @@
         <v>2026</v>
       </c>
       <c r="H55">
-        <v>2.727804347236687</v>
+        <v>2.971249183230392</v>
       </c>
       <c r="I55">
         <v>2025</v>
@@ -3278,7 +3278,7 @@
         <v>2015</v>
       </c>
       <c r="O55">
-        <v>7.025</v>
+        <v>7.23</v>
       </c>
     </row>
     <row r="56">
@@ -3307,10 +3307,10 @@
         </is>
       </c>
       <c r="G56">
-        <v>2086</v>
+        <v>2089</v>
       </c>
       <c r="H56">
-        <v>1.135649383569506</v>
+        <v>1.125993835819224</v>
       </c>
       <c r="I56">
         <v>2025</v>
@@ -3335,7 +3335,7 @@
         <v>2015</v>
       </c>
       <c r="O56">
-        <v>33.31</v>
+        <v>33.245</v>
       </c>
     </row>
     <row r="57">
@@ -3367,7 +3367,7 @@
         <v>2035</v>
       </c>
       <c r="H57">
-        <v>2.218626626665139</v>
+        <v>2.325472394592339</v>
       </c>
       <c r="I57">
         <v>2025</v>
@@ -3392,7 +3392,7 @@
         <v>2015</v>
       </c>
       <c r="O57">
-        <v>11.9</v>
+        <v>12.02</v>
       </c>
     </row>
     <row r="58">
@@ -3421,7 +3421,7 @@
         </is>
       </c>
       <c r="H58">
-        <v>-0.5835487311161757</v>
+        <v>-0.5831645129158318</v>
       </c>
       <c r="I58">
         <v>2025</v>
@@ -3446,7 +3446,7 @@
         <v>2015</v>
       </c>
       <c r="O58">
-        <v>11.9</v>
+        <v>12.02</v>
       </c>
     </row>
     <row r="59">
@@ -3475,10 +3475,10 @@
         </is>
       </c>
       <c r="G59">
-        <v>2574</v>
+        <v>2600</v>
       </c>
       <c r="H59">
-        <v>0.1434468715290649</v>
+        <v>0.1418918918918905</v>
       </c>
       <c r="I59">
         <v>2025</v>
@@ -3503,7 +3503,7 @@
         <v>2015</v>
       </c>
       <c r="O59">
-        <v>33.21</v>
+        <v>33.145</v>
       </c>
     </row>
     <row r="60">
@@ -3532,7 +3532,7 @@
         </is>
       </c>
       <c r="H60">
-        <v>-1.190839734732737</v>
+        <v>-1.281096197620178</v>
       </c>
       <c r="I60">
         <v>2025</v>
@@ -3557,7 +3557,7 @@
         <v>2015</v>
       </c>
       <c r="O60">
-        <v>4.175</v>
+        <v>4.34</v>
       </c>
     </row>
     <row r="61">
@@ -3611,7 +3611,7 @@
         <v>2015</v>
       </c>
       <c r="O61">
-        <v>1.265</v>
+        <v>1.33</v>
       </c>
     </row>
     <row r="62">
@@ -3665,7 +3665,7 @@
         <v>2015</v>
       </c>
       <c r="O62">
-        <v>0.64</v>
+        <v>0.675</v>
       </c>
     </row>
     <row r="63">
@@ -3694,7 +3694,7 @@
         </is>
       </c>
       <c r="H63">
-        <v>-0.4453776651938398</v>
+        <v>-0.4777305174269116</v>
       </c>
       <c r="I63">
         <v>2025</v>
@@ -3719,7 +3719,7 @@
         <v>2015</v>
       </c>
       <c r="O63">
-        <v>5.265000000000001</v>
+        <v>5.45</v>
       </c>
     </row>
     <row r="64">
@@ -3751,7 +3751,7 @@
         <v>2023</v>
       </c>
       <c r="H64">
-        <v>2.707887180825716</v>
+        <v>2.980843263128079</v>
       </c>
       <c r="I64">
         <v>2025</v>
@@ -3776,7 +3776,7 @@
         <v>2015</v>
       </c>
       <c r="O64">
-        <v>5.33</v>
+        <v>5.52</v>
       </c>
     </row>
     <row r="65">
@@ -3805,10 +3805,10 @@
         </is>
       </c>
       <c r="G65">
-        <v>2073</v>
+        <v>2076</v>
       </c>
       <c r="H65">
-        <v>0.852143578470708</v>
+        <v>0.857154425616045</v>
       </c>
       <c r="I65">
         <v>2025</v>
@@ -3833,7 +3833,7 @@
         <v>2015</v>
       </c>
       <c r="O65">
-        <v>14.27</v>
+        <v>14.32</v>
       </c>
     </row>
     <row r="66">
@@ -3887,7 +3887,7 @@
         <v>2015</v>
       </c>
       <c r="O66">
-        <v>0.465</v>
+        <v>0.485</v>
       </c>
     </row>
     <row r="67">
@@ -3916,7 +3916,7 @@
         </is>
       </c>
       <c r="H67">
-        <v>-1.310496112550908</v>
+        <v>-1.308330248056276</v>
       </c>
       <c r="I67">
         <v>2025</v>
@@ -3941,7 +3941,7 @@
         <v>2015</v>
       </c>
       <c r="O67">
-        <v>31.765</v>
+        <v>31.7</v>
       </c>
     </row>
     <row r="68">
@@ -3995,7 +3995,7 @@
         <v>2015</v>
       </c>
       <c r="O68">
-        <v>0.64</v>
+        <v>0.675</v>
       </c>
     </row>
     <row r="69">
@@ -4027,7 +4027,7 @@
         <v>2027</v>
       </c>
       <c r="H69">
-        <v>4.529643057599236</v>
+        <v>4.778620103613849</v>
       </c>
       <c r="I69">
         <v>2025</v>
@@ -4052,7 +4052,7 @@
         <v>2015</v>
       </c>
       <c r="O69">
-        <v>15.7</v>
+        <v>15.705</v>
       </c>
     </row>
     <row r="70">
@@ -4084,13 +4084,13 @@
         <v>2023</v>
       </c>
       <c r="H70">
-        <v>5.722312008143362</v>
+        <v>6.29421872153674</v>
       </c>
       <c r="I70">
         <v>2025</v>
       </c>
       <c r="J70">
-        <v>1.54</v>
+        <v>1.5</v>
       </c>
       <c r="K70">
         <v>15.9</v>
@@ -4109,7 +4109,7 @@
         <v>2015</v>
       </c>
       <c r="O70">
-        <v>11.025</v>
+        <v>11.17</v>
       </c>
     </row>
     <row r="71">
@@ -4186,7 +4186,7 @@
         <v>2022</v>
       </c>
       <c r="H72">
-        <v>0.5283300033300037</v>
+        <v>0.5863636363636374</v>
       </c>
       <c r="I72">
         <v>2025</v>
@@ -4211,7 +4211,7 @@
         <v>2015</v>
       </c>
       <c r="O72">
-        <v>1.955</v>
+        <v>2.055</v>
       </c>
     </row>
     <row r="73">
@@ -4265,7 +4265,7 @@
         <v>2015</v>
       </c>
       <c r="O73">
-        <v>0.35</v>
+        <v>0.37</v>
       </c>
     </row>
     <row r="74">
@@ -4364,7 +4364,7 @@
         <v>2015</v>
       </c>
       <c r="O75">
-        <v>0.35</v>
+        <v>0.37</v>
       </c>
     </row>
     <row r="76">
@@ -4418,7 +4418,7 @@
         <v>2015</v>
       </c>
       <c r="O76">
-        <v>1.325</v>
+        <v>1.39</v>
       </c>
     </row>
     <row r="77">
@@ -4472,7 +4472,7 @@
         <v>2015</v>
       </c>
       <c r="O77">
-        <v>0.35</v>
+        <v>0.37</v>
       </c>
     </row>
     <row r="78">
@@ -4645,7 +4645,7 @@
         </is>
       </c>
       <c r="H81">
-        <v>-0.5855053683820813</v>
+        <v>-0.5825990373935582</v>
       </c>
       <c r="I81">
         <v>2025</v>
@@ -4670,7 +4670,7 @@
         <v>2015</v>
       </c>
       <c r="O81">
-        <v>30.72</v>
+        <v>30.645</v>
       </c>
     </row>
     <row r="82">
@@ -4702,7 +4702,7 @@
         <v>2023</v>
       </c>
       <c r="H82">
-        <v>5.184417442813199</v>
+        <v>5.710435420969259</v>
       </c>
       <c r="I82">
         <v>2025</v>
@@ -4727,7 +4727,7 @@
         <v>2015</v>
       </c>
       <c r="O82">
-        <v>7.315</v>
+        <v>7.515000000000001</v>
       </c>
     </row>
     <row r="83">
@@ -4759,7 +4759,7 @@
         <v>2021</v>
       </c>
       <c r="H83">
-        <v>6.299148905212436</v>
+        <v>7.031597231382048</v>
       </c>
       <c r="I83">
         <v>2025</v>
@@ -4784,7 +4784,7 @@
         <v>2015</v>
       </c>
       <c r="O83">
-        <v>5.265000000000001</v>
+        <v>5.45</v>
       </c>
     </row>
     <row r="84">
@@ -4858,10 +4858,10 @@
         </is>
       </c>
       <c r="G85">
-        <v>2030</v>
+        <v>2031</v>
       </c>
       <c r="H85">
-        <v>3.050803976794103</v>
+        <v>3.209324355016082</v>
       </c>
       <c r="I85">
         <v>2025</v>
@@ -4886,7 +4886,7 @@
         <v>2015</v>
       </c>
       <c r="O85">
-        <v>13.035</v>
+        <v>13.12</v>
       </c>
     </row>
     <row r="86">
@@ -4915,7 +4915,7 @@
         </is>
       </c>
       <c r="H86">
-        <v>-1.2061708719308</v>
+        <v>-1.326896872354101</v>
       </c>
       <c r="I86">
         <v>2025</v>
@@ -4940,7 +4940,7 @@
         <v>2015</v>
       </c>
       <c r="O86">
-        <v>2.47</v>
+        <v>2.585</v>
       </c>
     </row>
     <row r="87">
@@ -4969,7 +4969,7 @@
         </is>
       </c>
       <c r="H87">
-        <v>-0.08565392354124697</v>
+        <v>-0.08450704225352013</v>
       </c>
       <c r="I87">
         <v>2025</v>
@@ -4994,7 +4994,7 @@
         <v>2015</v>
       </c>
       <c r="O87">
-        <v>25.2</v>
+        <v>25.085</v>
       </c>
     </row>
     <row r="88">
@@ -5071,7 +5071,7 @@
         <v>2025</v>
       </c>
       <c r="H89">
-        <v>0.8819139713915263</v>
+        <v>0.9785819327731105</v>
       </c>
       <c r="I89">
         <v>2025</v>
@@ -5096,7 +5096,7 @@
         <v>2015</v>
       </c>
       <c r="O89">
-        <v>2.785</v>
+        <v>2.915</v>
       </c>
     </row>
     <row r="90">
@@ -5150,7 +5150,7 @@
         <v>2015</v>
       </c>
       <c r="O90">
-        <v>33.59</v>
+        <v>33.535</v>
       </c>
     </row>
     <row r="91">
@@ -5204,7 +5204,7 @@
         <v>2015</v>
       </c>
       <c r="O91">
-        <v>0.64</v>
+        <v>0.675</v>
       </c>
     </row>
     <row r="92">
@@ -5303,7 +5303,7 @@
         <v>2015</v>
       </c>
       <c r="O93">
-        <v>0.64</v>
+        <v>0.675</v>
       </c>
     </row>
     <row r="94">
@@ -5335,7 +5335,7 @@
         <v>2021</v>
       </c>
       <c r="H94">
-        <v>0.8248235098235085</v>
+        <v>0.9175602175602166</v>
       </c>
       <c r="I94">
         <v>2025</v>
@@ -5360,7 +5360,7 @@
         <v>2015</v>
       </c>
       <c r="O94">
-        <v>2.08</v>
+        <v>2.18</v>
       </c>
     </row>
     <row r="95">
@@ -5434,10 +5434,10 @@
         </is>
       </c>
       <c r="G96">
-        <v>2410</v>
+        <v>2416</v>
       </c>
       <c r="H96">
-        <v>0.3023289490527389</v>
+        <v>0.3057351867240826</v>
       </c>
       <c r="I96">
         <v>2025</v>
@@ -5462,7 +5462,7 @@
         <v>2015</v>
       </c>
       <c r="O96">
-        <v>61.565</v>
+        <v>61.64</v>
       </c>
     </row>
     <row r="97">
@@ -5539,7 +5539,7 @@
         <v>2021</v>
       </c>
       <c r="H98">
-        <v>2.368386154179498</v>
+        <v>2.637856400135811</v>
       </c>
       <c r="I98">
         <v>2025</v>
@@ -5564,7 +5564,7 @@
         <v>2015</v>
       </c>
       <c r="O98">
-        <v>2.85</v>
+        <v>2.985</v>
       </c>
     </row>
     <row r="99">
@@ -5596,7 +5596,7 @@
         <v>2018</v>
       </c>
       <c r="H99">
-        <v>3.351932520094283</v>
+        <v>3.741876007978951</v>
       </c>
       <c r="I99">
         <v>2025</v>
@@ -5621,7 +5621,7 @@
         <v>2015</v>
       </c>
       <c r="O99">
-        <v>2.725</v>
+        <v>2.85</v>
       </c>
     </row>
     <row r="100">
@@ -5653,7 +5653,7 @@
         <v>2025</v>
       </c>
       <c r="H100">
-        <v>2.314655960109093</v>
+        <v>2.555436332893561</v>
       </c>
       <c r="I100">
         <v>2025</v>
@@ -5678,7 +5678,7 @@
         <v>2015</v>
       </c>
       <c r="O100">
-        <v>4.51</v>
+        <v>4.685</v>
       </c>
     </row>
     <row r="101">
@@ -5707,7 +5707,7 @@
         </is>
       </c>
       <c r="H101">
-        <v>-0.1323943661971811</v>
+        <v>-0.130770735524257</v>
       </c>
       <c r="I101">
         <v>2025</v>
@@ -5732,7 +5732,7 @@
         <v>2015</v>
       </c>
       <c r="O101">
-        <v>25.85</v>
+        <v>25.735</v>
       </c>
     </row>
     <row r="102">
@@ -5806,10 +5806,10 @@
         </is>
       </c>
       <c r="G103">
-        <v>2092</v>
+        <v>2096</v>
       </c>
       <c r="H103">
-        <v>0.6040320242301391</v>
+        <v>0.6111282615375699</v>
       </c>
       <c r="I103">
         <v>2025</v>
@@ -5834,7 +5834,7 @@
         <v>2015</v>
       </c>
       <c r="O103">
-        <v>12.87</v>
+        <v>12.965</v>
       </c>
     </row>
     <row r="104">
@@ -5866,7 +5866,7 @@
         <v>2019</v>
       </c>
       <c r="H104">
-        <v>1.64466477966478</v>
+        <v>1.836165223665222</v>
       </c>
       <c r="I104">
         <v>2025</v>
@@ -5891,7 +5891,7 @@
         <v>2015</v>
       </c>
       <c r="O104">
-        <v>2.335</v>
+        <v>2.445</v>
       </c>
     </row>
     <row r="105">
@@ -5965,7 +5965,7 @@
         </is>
       </c>
       <c r="H106">
-        <v>-1.481234857631203</v>
+        <v>-1.499643485378478</v>
       </c>
       <c r="I106">
         <v>2025</v>
@@ -5990,7 +5990,7 @@
         <v>2015</v>
       </c>
       <c r="O106">
-        <v>68.375</v>
+        <v>68.45</v>
       </c>
     </row>
     <row r="107">
@@ -6019,10 +6019,10 @@
         </is>
       </c>
       <c r="G107">
-        <v>2129</v>
+        <v>2132</v>
       </c>
       <c r="H107">
-        <v>0.2782640466080778</v>
+        <v>0.294605840658474</v>
       </c>
       <c r="I107">
         <v>2025</v>
@@ -6047,7 +6047,7 @@
         <v>2015</v>
       </c>
       <c r="O107">
-        <v>7.385</v>
+        <v>7.59</v>
       </c>
     </row>
     <row r="108">
@@ -6101,7 +6101,7 @@
         <v>2015</v>
       </c>
       <c r="O108">
-        <v>0.465</v>
+        <v>0.485</v>
       </c>
     </row>
     <row r="109">
@@ -6130,7 +6130,7 @@
         </is>
       </c>
       <c r="H109">
-        <v>-1.012125481504887</v>
+        <v>-1.025032549344344</v>
       </c>
       <c r="I109">
         <v>2025</v>
@@ -6155,7 +6155,7 @@
         <v>2015</v>
       </c>
       <c r="O109">
-        <v>64.44499999999999</v>
+        <v>64.52</v>
       </c>
     </row>
     <row r="110">
@@ -6229,10 +6229,10 @@
         </is>
       </c>
       <c r="G111">
-        <v>2200</v>
+        <v>2214</v>
       </c>
       <c r="H111">
-        <v>0.3038772842117652</v>
+        <v>0.2985606217259431</v>
       </c>
       <c r="I111">
         <v>2025</v>
@@ -6257,7 +6257,7 @@
         <v>2015</v>
       </c>
       <c r="O111">
-        <v>17.94</v>
+        <v>17.88</v>
       </c>
     </row>
     <row r="112">
@@ -6286,10 +6286,10 @@
         </is>
       </c>
       <c r="G112">
-        <v>2063</v>
+        <v>2064</v>
       </c>
       <c r="H112">
-        <v>2.287401966569794</v>
+        <v>2.301806461657992</v>
       </c>
       <c r="I112">
         <v>2025</v>
@@ -6314,7 +6314,7 @@
         <v>2015</v>
       </c>
       <c r="O112">
-        <v>55.605</v>
+        <v>55.67</v>
       </c>
     </row>
     <row r="113">
@@ -6343,7 +6343,7 @@
         </is>
       </c>
       <c r="H113">
-        <v>-2.619977939130942</v>
+        <v>-2.610621855697104</v>
       </c>
       <c r="I113">
         <v>2025</v>
@@ -6368,7 +6368,7 @@
         <v>2015</v>
       </c>
       <c r="O113">
-        <v>24.745</v>
+        <v>24.62</v>
       </c>
     </row>
     <row r="114">
@@ -6397,10 +6397,10 @@
         </is>
       </c>
       <c r="G114">
-        <v>2058</v>
+        <v>2059</v>
       </c>
       <c r="H114">
-        <v>0.3809822134387361</v>
+        <v>0.4173244871070949</v>
       </c>
       <c r="I114">
         <v>2025</v>
@@ -6425,7 +6425,7 @@
         <v>2015</v>
       </c>
       <c r="O114">
-        <v>3.9</v>
+        <v>4.065</v>
       </c>
     </row>
     <row r="115">
@@ -6547,7 +6547,7 @@
         <v>2021</v>
       </c>
       <c r="H117">
-        <v>2.839034365617183</v>
+        <v>3.16110717412962</v>
       </c>
       <c r="I117">
         <v>2025</v>
@@ -6572,7 +6572,7 @@
         <v>2015</v>
       </c>
       <c r="O117">
-        <v>3.375</v>
+        <v>3.525</v>
       </c>
     </row>
     <row r="118">
@@ -6604,7 +6604,7 @@
         <v>2026</v>
       </c>
       <c r="H118">
-        <v>1.698113371152712</v>
+        <v>1.870559876017106</v>
       </c>
       <c r="I118">
         <v>2025</v>
@@ -6629,7 +6629,7 @@
         <v>2015</v>
       </c>
       <c r="O118">
-        <v>4.24</v>
+        <v>4.41</v>
       </c>
     </row>
     <row r="119">
@@ -6658,7 +6658,7 @@
         </is>
       </c>
       <c r="H119">
-        <v>-0.7796152789569362</v>
+        <v>-0.7725780204701238</v>
       </c>
       <c r="I119">
         <v>2025</v>
@@ -6683,7 +6683,7 @@
         <v>2015</v>
       </c>
       <c r="O119">
-        <v>12.87</v>
+        <v>12.965</v>
       </c>
     </row>
     <row r="120">
@@ -6715,7 +6715,7 @@
         <v>2025</v>
       </c>
       <c r="H120">
-        <v>1.132278343861162</v>
+        <v>1.253814130915526</v>
       </c>
       <c r="I120">
         <v>2025</v>
@@ -6740,7 +6740,7 @@
         <v>2015</v>
       </c>
       <c r="O120">
-        <v>3.05</v>
+        <v>3.185</v>
       </c>
     </row>
     <row r="121">
@@ -6772,7 +6772,7 @@
         <v>2036</v>
       </c>
       <c r="H121">
-        <v>1.124362375093091</v>
+        <v>1.226279530936637</v>
       </c>
       <c r="I121">
         <v>2025</v>
@@ -6797,7 +6797,7 @@
         <v>2015</v>
       </c>
       <c r="O121">
-        <v>5.195</v>
+        <v>5.385</v>
       </c>
     </row>
     <row r="122">
@@ -6829,7 +6829,7 @@
         <v>2028</v>
       </c>
       <c r="H122">
-        <v>3.037345254112586</v>
+        <v>3.256507579504171</v>
       </c>
       <c r="I122">
         <v>2025</v>
@@ -6854,7 +6854,7 @@
         <v>2015</v>
       </c>
       <c r="O122">
-        <v>10.015</v>
+        <v>10.185</v>
       </c>
     </row>
     <row r="123">
@@ -6883,7 +6883,7 @@
         </is>
       </c>
       <c r="G123">
-        <v>2263</v>
+        <v>2271</v>
       </c>
       <c r="H123">
         <v>0.3513513513513516</v>
@@ -6911,7 +6911,7 @@
         <v>2015</v>
       </c>
       <c r="O123">
-        <v>38.26</v>
+        <v>38.24</v>
       </c>
     </row>
     <row r="124">
@@ -6965,7 +6965,7 @@
         <v>2015</v>
       </c>
       <c r="O124">
-        <v>0.35</v>
+        <v>0.37</v>
       </c>
     </row>
     <row r="125">
@@ -7019,7 +7019,7 @@
         <v>2015</v>
       </c>
       <c r="O125">
-        <v>0.465</v>
+        <v>0.485</v>
       </c>
     </row>
     <row r="126">
@@ -7051,13 +7051,13 @@
         <v>2023</v>
       </c>
       <c r="H126">
-        <v>2.446226629874667</v>
+        <v>2.499916697939145</v>
       </c>
       <c r="I126">
         <v>2025</v>
       </c>
       <c r="J126">
-        <v>1.9</v>
+        <v>2.07</v>
       </c>
       <c r="K126">
         <v>5.5</v>
@@ -7076,7 +7076,7 @@
         <v>2015</v>
       </c>
       <c r="O126">
-        <v>3.51</v>
+        <v>3.66</v>
       </c>
     </row>
     <row r="127">
@@ -7127,7 +7127,7 @@
         <v>2015</v>
       </c>
       <c r="O127">
-        <v>0.8300000000000001</v>
+        <v>0.87</v>
       </c>
     </row>
     <row r="128">
@@ -7204,7 +7204,7 @@
         <v>2020</v>
       </c>
       <c r="H129">
-        <v>5.940076324567275</v>
+        <v>6.659700679657911</v>
       </c>
       <c r="I129">
         <v>2025</v>
@@ -7229,7 +7229,7 @@
         <v>2015</v>
       </c>
       <c r="O129">
-        <v>4.92</v>
+        <v>5.105</v>
       </c>
     </row>
     <row r="130">
@@ -7303,10 +7303,10 @@
         </is>
       </c>
       <c r="G131">
-        <v>2056</v>
+        <v>2057</v>
       </c>
       <c r="H131">
-        <v>2.405792093463327</v>
+        <v>2.406613291373566</v>
       </c>
       <c r="I131">
         <v>2025</v>
@@ -7331,7 +7331,7 @@
         <v>2015</v>
       </c>
       <c r="O131">
-        <v>46.905</v>
+        <v>46.945</v>
       </c>
     </row>
     <row r="132">
@@ -7360,7 +7360,7 @@
         </is>
       </c>
       <c r="H132">
-        <v>-7.532840442939658</v>
+        <v>-7.551237451924718</v>
       </c>
       <c r="I132">
         <v>2025</v>
@@ -7385,7 +7385,7 @@
         <v>2015</v>
       </c>
       <c r="O132">
-        <v>6.805</v>
+        <v>7.015000000000001</v>
       </c>
     </row>
     <row r="133">
@@ -7414,10 +7414,10 @@
         </is>
       </c>
       <c r="G133">
-        <v>2061</v>
+        <v>2064</v>
       </c>
       <c r="H133">
-        <v>1.191687593997906</v>
+        <v>1.185536573098489</v>
       </c>
       <c r="I133">
         <v>2025</v>
@@ -7442,7 +7442,7 @@
         <v>2015</v>
       </c>
       <c r="O133">
-        <v>17.155</v>
+        <v>17.115</v>
       </c>
     </row>
     <row r="134">
@@ -7496,7 +7496,7 @@
         <v>2015</v>
       </c>
       <c r="O134">
-        <v>34.36</v>
+        <v>34.315</v>
       </c>
     </row>
     <row r="135">
@@ -7550,7 +7550,7 @@
         <v>2015</v>
       </c>
       <c r="O135">
-        <v>43.145</v>
+        <v>43.155</v>
       </c>
     </row>
     <row r="136">
@@ -7582,7 +7582,7 @@
         <v>2042</v>
       </c>
       <c r="H136">
-        <v>0.4957526391736934</v>
+        <v>0.5467801857585158</v>
       </c>
       <c r="I136">
         <v>2025</v>
@@ -7607,7 +7607,7 @@
         <v>2015</v>
       </c>
       <c r="O136">
-        <v>3.375</v>
+        <v>3.525</v>
       </c>
     </row>
     <row r="137">
@@ -7639,7 +7639,7 @@
         <v>2019</v>
       </c>
       <c r="H137">
-        <v>4.990910268848799</v>
+        <v>5.530414435683125</v>
       </c>
       <c r="I137">
         <v>2025</v>
@@ -7664,7 +7664,7 @@
         <v>2015</v>
       </c>
       <c r="O137">
-        <v>5.47</v>
+        <v>5.665</v>
       </c>
     </row>
     <row r="138">
@@ -7693,7 +7693,7 @@
         </is>
       </c>
       <c r="H138">
-        <v>-3.15233843585379</v>
+        <v>-3.190078343734321</v>
       </c>
       <c r="I138">
         <v>2025</v>
@@ -7718,7 +7718,7 @@
         <v>2015</v>
       </c>
       <c r="O138">
-        <v>64.77500000000001</v>
+        <v>64.85499999999999</v>
       </c>
     </row>
     <row r="139">
@@ -7747,10 +7747,10 @@
         </is>
       </c>
       <c r="G139">
-        <v>2123</v>
+        <v>2128</v>
       </c>
       <c r="H139">
-        <v>0.370664009452068</v>
+        <v>0.3823976349993927</v>
       </c>
       <c r="I139">
         <v>2025</v>
@@ -7775,7 +7775,7 @@
         <v>2015</v>
       </c>
       <c r="O139">
-        <v>10.165</v>
+        <v>10.335</v>
       </c>
     </row>
     <row r="140">
@@ -7829,7 +7829,7 @@
         <v>2015</v>
       </c>
       <c r="O140">
-        <v>0.71</v>
+        <v>0.74</v>
       </c>
     </row>
     <row r="141">
@@ -7883,7 +7883,7 @@
         <v>2015</v>
       </c>
       <c r="O141">
-        <v>0.535</v>
+        <v>0.555</v>
       </c>
     </row>
     <row r="142">
@@ -7982,7 +7982,7 @@
         <v>2015</v>
       </c>
       <c r="O143">
-        <v>0.465</v>
+        <v>0.485</v>
       </c>
     </row>
     <row r="144">
@@ -8011,10 +8011,10 @@
         </is>
       </c>
       <c r="G144">
-        <v>2111</v>
+        <v>2114</v>
       </c>
       <c r="H144">
-        <v>0.9140873750462788</v>
+        <v>0.9121621621621643</v>
       </c>
       <c r="I144">
         <v>2025</v>
@@ -8039,7 +8039,7 @@
         <v>2015</v>
       </c>
       <c r="O144">
-        <v>38.56</v>
+        <v>38.54</v>
       </c>
     </row>
     <row r="145">
@@ -8093,7 +8093,7 @@
         <v>2015</v>
       </c>
       <c r="O145">
-        <v>0.8300000000000001</v>
+        <v>0.87</v>
       </c>
     </row>
     <row r="146">
@@ -8122,7 +8122,7 @@
         </is>
       </c>
       <c r="H146">
-        <v>-1.320518526345825</v>
+        <v>-1.331940343303964</v>
       </c>
       <c r="I146">
         <v>2025</v>
@@ -8147,7 +8147,7 @@
         <v>2015</v>
       </c>
       <c r="O146">
-        <v>9.395</v>
+        <v>9.58</v>
       </c>
     </row>
     <row r="147">
@@ -8176,7 +8176,7 @@
         </is>
       </c>
       <c r="H147">
-        <v>-0.4491484635320262</v>
+        <v>-0.4462421325435031</v>
       </c>
       <c r="I147">
         <v>2025</v>
@@ -8201,7 +8201,7 @@
         <v>2015</v>
       </c>
       <c r="O147">
-        <v>29.97</v>
+        <v>29.875</v>
       </c>
     </row>
     <row r="148">
@@ -8230,16 +8230,16 @@
         </is>
       </c>
       <c r="G148">
-        <v>2071</v>
+        <v>2073</v>
       </c>
       <c r="H148">
-        <v>1.37098550369883</v>
+        <v>1.365989452032159</v>
       </c>
       <c r="I148">
         <v>2025</v>
       </c>
       <c r="J148">
-        <v>28.34</v>
+        <v>28.26</v>
       </c>
       <c r="K148">
         <v>38</v>
@@ -8258,7 +8258,7 @@
         <v>2015</v>
       </c>
       <c r="O148">
-        <v>30.53</v>
+        <v>30.455</v>
       </c>
     </row>
     <row r="149">
@@ -8335,7 +8335,7 @@
         <v>2029</v>
       </c>
       <c r="H150">
-        <v>3.015915103104814</v>
+        <v>3.215650247097523</v>
       </c>
       <c r="I150">
         <v>2025</v>
@@ -8360,7 +8360,7 @@
         <v>2015</v>
       </c>
       <c r="O150">
-        <v>10.87</v>
+        <v>11.02</v>
       </c>
     </row>
     <row r="151">
@@ -8392,7 +8392,7 @@
         <v>2023</v>
       </c>
       <c r="H151">
-        <v>1.68865197023479</v>
+        <v>1.873218702951675</v>
       </c>
       <c r="I151">
         <v>2025</v>
@@ -8417,7 +8417,7 @@
         <v>2015</v>
       </c>
       <c r="O151">
-        <v>3.175</v>
+        <v>3.32</v>
       </c>
     </row>
     <row r="152">
@@ -8446,13 +8446,13 @@
         </is>
       </c>
       <c r="H152">
-        <v>-0.6486486486486485</v>
+        <v>-0.2229729729729712</v>
       </c>
       <c r="I152">
         <v>2025</v>
       </c>
       <c r="J152">
-        <v>48.6</v>
+        <v>45.45</v>
       </c>
       <c r="K152">
         <v>43.8</v>
@@ -8471,7 +8471,7 @@
         <v>2015</v>
       </c>
       <c r="O152">
-        <v>36.105</v>
+        <v>36.07</v>
       </c>
     </row>
     <row r="153">
@@ -8624,7 +8624,7 @@
         <v>2015</v>
       </c>
       <c r="O155">
-        <v>0.535</v>
+        <v>0.555</v>
       </c>
     </row>
     <row r="156">
@@ -8701,7 +8701,7 @@
         <v>2021</v>
       </c>
       <c r="H157">
-        <v>3.67865727169661</v>
+        <v>4.091728762685992</v>
       </c>
       <c r="I157">
         <v>2025</v>
@@ -8726,7 +8726,7 @@
         <v>2015</v>
       </c>
       <c r="O157">
-        <v>4.105</v>
+        <v>4.275</v>
       </c>
     </row>
     <row r="158">
@@ -8800,10 +8800,10 @@
         </is>
       </c>
       <c r="G159">
-        <v>2250</v>
+        <v>2255</v>
       </c>
       <c r="H159">
-        <v>0.4024065161051453</v>
+        <v>0.4045168456127357</v>
       </c>
       <c r="I159">
         <v>2025</v>
@@ -8828,7 +8828,7 @@
         <v>2015</v>
       </c>
       <c r="O159">
-        <v>43.545</v>
+        <v>43.565</v>
       </c>
     </row>
     <row r="160">
@@ -8857,10 +8857,10 @@
         </is>
       </c>
       <c r="G160">
-        <v>2221</v>
+        <v>2225</v>
       </c>
       <c r="H160">
-        <v>0.5064542812430147</v>
+        <v>0.510382293762575</v>
       </c>
       <c r="I160">
         <v>2025</v>
@@ -8885,7 +8885,7 @@
         <v>2015</v>
       </c>
       <c r="O160">
-        <v>50.85</v>
+        <v>50.9</v>
       </c>
     </row>
     <row r="161">
@@ -9029,7 +9029,7 @@
         <v>2015</v>
       </c>
       <c r="O163">
-        <v>0.77</v>
+        <v>0.8100000000000001</v>
       </c>
     </row>
     <row r="164">
@@ -9061,7 +9061,7 @@
         <v>2024</v>
       </c>
       <c r="H164">
-        <v>2.595565051018181</v>
+        <v>2.867658555115781</v>
       </c>
       <c r="I164">
         <v>2025</v>
@@ -9086,7 +9086,7 @@
         <v>2015</v>
       </c>
       <c r="O164">
-        <v>4.51</v>
+        <v>4.685</v>
       </c>
     </row>
     <row r="165">
@@ -9182,7 +9182,7 @@
         <v>2015</v>
       </c>
       <c r="O166">
-        <v>1.825</v>
+        <v>1.92</v>
       </c>
     </row>
     <row r="167">
@@ -9211,7 +9211,7 @@
         </is>
       </c>
       <c r="H167">
-        <v>-0.4125955238462297</v>
+        <v>-0.4068125120663467</v>
       </c>
       <c r="I167">
         <v>2025</v>
@@ -9236,7 +9236,7 @@
         <v>2015</v>
       </c>
       <c r="O167">
-        <v>14.69</v>
+        <v>14.725</v>
       </c>
     </row>
     <row r="168">
@@ -9268,7 +9268,7 @@
         <v>2022</v>
       </c>
       <c r="H168">
-        <v>1.517164779664782</v>
+        <v>1.69330808080808</v>
       </c>
       <c r="I168">
         <v>2025</v>
@@ -9293,7 +9293,7 @@
         <v>2015</v>
       </c>
       <c r="O168">
-        <v>2.205</v>
+        <v>2.32</v>
       </c>
     </row>
     <row r="169">
@@ -9322,10 +9322,10 @@
         </is>
       </c>
       <c r="G169">
-        <v>2040</v>
+        <v>2041</v>
       </c>
       <c r="H169">
-        <v>1.708494297125185</v>
+        <v>1.781241974667017</v>
       </c>
       <c r="I169">
         <v>2025</v>
@@ -9350,7 +9350,7 @@
         <v>2015</v>
       </c>
       <c r="O169">
-        <v>11.58</v>
+        <v>11.71</v>
       </c>
     </row>
     <row r="170">
@@ -9379,7 +9379,7 @@
         </is>
       </c>
       <c r="H170">
-        <v>-3.579782837828149</v>
+        <v>-3.612974704378593</v>
       </c>
       <c r="I170">
         <v>2025</v>
@@ -9404,7 +9404,7 @@
         <v>2015</v>
       </c>
       <c r="O170">
-        <v>42.335</v>
+        <v>42.345</v>
       </c>
     </row>
     <row r="171">
@@ -9433,10 +9433,10 @@
         </is>
       </c>
       <c r="G171">
-        <v>2053</v>
+        <v>2056</v>
       </c>
       <c r="H171">
-        <v>1.608831046204725</v>
+        <v>1.587979034135515</v>
       </c>
       <c r="I171">
         <v>2025</v>
@@ -9461,7 +9461,7 @@
         <v>2015</v>
       </c>
       <c r="O171">
-        <v>21.025</v>
+        <v>20.915</v>
       </c>
     </row>
     <row r="172">
@@ -9490,13 +9490,13 @@
         </is>
       </c>
       <c r="H172">
-        <v>-0.3778089194429753</v>
+        <v>-0.4177105498241744</v>
       </c>
       <c r="I172">
         <v>2025</v>
       </c>
       <c r="J172">
-        <v>70.21000000000001</v>
+        <v>70.42</v>
       </c>
       <c r="K172">
         <v>67.90000000000001</v>
@@ -9515,7 +9515,7 @@
         <v>2015</v>
       </c>
       <c r="O172">
-        <v>61.015</v>
+        <v>61.095</v>
       </c>
     </row>
     <row r="173">
@@ -9544,7 +9544,7 @@
         </is>
       </c>
       <c r="H173">
-        <v>-0.7365975564605691</v>
+        <v>-0.7351351351351354</v>
       </c>
       <c r="I173">
         <v>2025</v>
@@ -9569,7 +9569,7 @@
         <v>2015</v>
       </c>
       <c r="O173">
-        <v>32.245</v>
+        <v>32.18</v>
       </c>
     </row>
   </sheetData>

</xml_diff>